<commit_message>
Merge dataset, rerun embeddings and finalize other datasets for 50% presentation
</commit_message>
<xml_diff>
--- a/Dataset/Tagged_POS.xlsx
+++ b/Dataset/Tagged_POS.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[(b'anak', 'NOUN'), (b'sa', 'PART'), (b'bugoon', 'NOUN')]</t>
+          <t>[(b'anak', 'NOUN'), (b'sa', 'PART'), (b'bugoon', 'ADJ')]</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>[(b'klaro', 'ADJ'), (b'kaayo', 'NOUN'), (b'sa', 'PART'), (b'patern', 'NOUN')]</t>
+          <t>[(b'klaro', 'ADJ'), (b'kaayo', 'ADV'), (b'sa', 'PART'), (b'patern', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>[(b'agi', 'VERB'), (b'sa', 'PART'), (b'bangag', 'VERB'), (b'sa', 'PART'), (b'dagom', 'NOUN')]</t>
+          <t>[(b'agi', 'ADJ'), (b'sa', 'PART'), (b'bangag', 'VERB'), (b'sa', 'PART'), (b'dagom', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>[(b'karaang', 'ADJ'), (b'damang', 'NOUN')]</t>
+          <t>[(b'karaang', 'ADJ'), (b'damang', 'VERB')]</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>[(b'ang', 'DET'), (b'dili', 'ADV'), (b'kaantos', 'NOUN'), (b'dili', 'ADV'), (b'masantos', 'ADJ')]</t>
+          <t>[(b'ang', 'DET'), (b'dili', 'ADV'), (b'kaantos', 'ADV'), (b'dili', 'ADV'), (b'masantos', 'ADJ')]</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>[(b'ang', 'DET'), (b'kalimot', 'NOUN'), (b'walay', 'ADV'), (b'gahom', 'NOUN')]</t>
+          <t>[(b'ang', 'DET'), (b'kalimot', 'ADV'), (b'walay', 'ADV'), (b'gahom', 'NOUN')]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix train split error
</commit_message>
<xml_diff>
--- a/Dataset/Tagged_POS.xlsx
+++ b/Dataset/Tagged_POS.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[(b'anak', 'NOUN'), (b'sa', 'PART'), (b'bugoon', 'ADJ')]</t>
+          <t>[(b'anak', 'NOUN'), (b'sa', 'PART'), (b'bugoon', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>[(b'klaro', 'ADJ'), (b'kaayo', 'ADV'), (b'sa', 'PART'), (b'patern', 'NOUN')]</t>
+          <t>[(b'klaro', 'ADJ'), (b'kaayo', 'NOUN'), (b'sa', 'PART'), (b'patern', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>[(b'agi', 'ADJ'), (b'sa', 'PART'), (b'bangag', 'VERB'), (b'sa', 'PART'), (b'dagom', 'NOUN')]</t>
+          <t>[(b'agi', 'VERB'), (b'sa', 'PART'), (b'bangag', 'VERB'), (b'sa', 'PART'), (b'dagom', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>[(b'karaang', 'ADJ'), (b'damang', 'VERB')]</t>
+          <t>[(b'karaang', 'ADJ'), (b'damang', 'NOUN')]</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>[(b'ang', 'DET'), (b'dili', 'ADV'), (b'kaantos', 'ADV'), (b'dili', 'ADV'), (b'masantos', 'ADJ')]</t>
+          <t>[(b'ang', 'DET'), (b'dili', 'ADV'), (b'kaantos', 'NOUN'), (b'dili', 'ADV'), (b'masantos', 'ADJ')]</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>[(b'ang', 'DET'), (b'kalimot', 'ADV'), (b'walay', 'ADV'), (b'gahom', 'NOUN')]</t>
+          <t>[(b'ang', 'DET'), (b'kalimot', 'NOUN'), (b'walay', 'ADV'), (b'gahom', 'NOUN')]</t>
         </is>
       </c>
     </row>

</xml_diff>